<commit_message>
feat(excelhasil): sesuaikan perhitungan excel  ΣM×w yang salah
</commit_message>
<xml_diff>
--- a/Fuzzy_AHP_3_Penilai_v9.xlsx
+++ b/Fuzzy_AHP_3_Penilai_v9.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29809"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29811"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\laragon\www\appSaringPramuka\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21799821-A901-4C47-B293-E4BB792000A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8C38D4E-3A36-42D0-956F-4248C5383AD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4596" yWindow="2400" windowWidth="17280" windowHeight="10188" firstSheet="3" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Input" sheetId="1" r:id="rId1"/>
@@ -669,8 +669,10 @@
     <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -708,8 +710,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1021,7 +1021,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="41" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="39"/>
@@ -1222,7 +1222,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="42" t="s">
         <v>30</v>
       </c>
       <c r="B1" s="39"/>
@@ -1273,10 +1273,18 @@
       <c r="D4" s="5">
         <v>5</v>
       </c>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
+      <c r="E4" s="5">
+        <v>3</v>
+      </c>
+      <c r="F4" s="5">
+        <v>4</v>
+      </c>
+      <c r="G4" s="5">
+        <v>4</v>
+      </c>
+      <c r="H4" s="5">
+        <v>88</v>
+      </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
@@ -1532,7 +1540,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="43" t="s">
         <v>31</v>
       </c>
       <c r="B1" s="39"/>
@@ -1577,16 +1585,24 @@
         <f>Input!B14</f>
         <v>David Kulian</v>
       </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
+      <c r="C4" s="5">
+        <v>4</v>
+      </c>
+      <c r="D4" s="5">
+        <v>4</v>
+      </c>
       <c r="E4" s="5">
         <v>3</v>
       </c>
       <c r="F4" s="5">
         <v>5</v>
       </c>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
+      <c r="G4" s="5">
+        <v>4</v>
+      </c>
+      <c r="H4" s="5">
+        <v>88</v>
+      </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
@@ -1842,7 +1858,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="44" t="s">
         <v>32</v>
       </c>
       <c r="B1" s="39"/>
@@ -1887,15 +1903,23 @@
         <f>Input!B14</f>
         <v>David Kulian</v>
       </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
+      <c r="C4" s="5">
+        <v>3</v>
+      </c>
+      <c r="D4" s="5">
+        <v>4</v>
+      </c>
+      <c r="E4" s="5">
+        <v>5</v>
+      </c>
+      <c r="F4" s="5">
+        <v>4</v>
+      </c>
       <c r="G4" s="5">
         <v>4</v>
       </c>
       <c r="H4" s="5">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
@@ -2152,7 +2176,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="46" t="s">
         <v>33</v>
       </c>
       <c r="B1" s="39"/>
@@ -2164,7 +2188,7 @@
       <c r="H1" s="39"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="45" t="s">
         <v>34</v>
       </c>
       <c r="B2" s="39"/>
@@ -2211,19 +2235,19 @@
       </c>
       <c r="C5" s="13">
         <f>AVERAGE('Penilai 1'!C4,'Penilai 2'!C4,'Penilai 3'!C4)</f>
-        <v>4</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="D5" s="13">
         <f>AVERAGE('Penilai 1'!D4,'Penilai 2'!D4,'Penilai 3'!D4)</f>
-        <v>5</v>
+        <v>4.333333333333333</v>
       </c>
       <c r="E5" s="13">
         <f>AVERAGE('Penilai 1'!E4,'Penilai 2'!E4,'Penilai 3'!E4)</f>
-        <v>3</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F5" s="13">
         <f>AVERAGE('Penilai 1'!F4,'Penilai 2'!F4,'Penilai 3'!F4)</f>
-        <v>5</v>
+        <v>4.333333333333333</v>
       </c>
       <c r="G5" s="13">
         <f>AVERAGE('Penilai 1'!G4,'Penilai 2'!G4,'Penilai 3'!G4)</f>
@@ -2231,7 +2255,7 @@
       </c>
       <c r="H5" s="13">
         <f>AVERAGE('Penilai 1'!H4,'Penilai 2'!H4,'Penilai 3'!H4)</f>
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
@@ -2550,7 +2574,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="46" t="s">
         <v>35</v>
       </c>
       <c r="B1" s="39"/>
@@ -2565,15 +2589,15 @@
       <c r="K1" s="39"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3" s="45" t="s">
+      <c r="A3" s="47" t="s">
         <v>36</v>
       </c>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
+      <c r="E3" s="48"/>
+      <c r="F3" s="48"/>
+      <c r="G3" s="48"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="14"/>
@@ -2765,15 +2789,15 @@
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" s="52" t="s">
+      <c r="A12" s="54" t="s">
         <v>37</v>
       </c>
-      <c r="B12" s="53"/>
-      <c r="C12" s="53"/>
-      <c r="D12" s="53"/>
-      <c r="E12" s="53"/>
-      <c r="F12" s="53"/>
-      <c r="G12" s="53"/>
+      <c r="B12" s="55"/>
+      <c r="C12" s="55"/>
+      <c r="D12" s="55"/>
+      <c r="E12" s="55"/>
+      <c r="F12" s="55"/>
+      <c r="G12" s="55"/>
     </row>
     <row r="13" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="16" t="s">
@@ -2878,15 +2902,15 @@
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="47" t="s">
+      <c r="A22" s="49" t="s">
         <v>41</v>
       </c>
-      <c r="B22" s="48"/>
-      <c r="C22" s="48"/>
-      <c r="D22" s="48"/>
-      <c r="E22" s="48"/>
-      <c r="F22" s="48"/>
-      <c r="G22" s="48"/>
+      <c r="B22" s="50"/>
+      <c r="C22" s="50"/>
+      <c r="D22" s="50"/>
+      <c r="E22" s="50"/>
+      <c r="F22" s="50"/>
+      <c r="G22" s="50"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="20" t="s">
@@ -3016,12 +3040,12 @@
       <c r="A35" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="B35" s="49" t="str">
+      <c r="B35" s="51" t="str">
         <f>IF(B34&lt;=0.1,"KONSISTEN","TIDAK KONSISTEN")</f>
         <v>KONSISTEN</v>
       </c>
-      <c r="C35" s="50"/>
-      <c r="D35" s="51"/>
+      <c r="C35" s="52"/>
+      <c r="D35" s="53"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -3045,7 +3069,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:27" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="46" t="s">
         <v>49</v>
       </c>
       <c r="B1" s="39"/>
@@ -3069,27 +3093,27 @@
       <c r="T1" s="39"/>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="A3" s="59" t="s">
+      <c r="A3" s="61" t="s">
         <v>50</v>
       </c>
-      <c r="B3" s="60"/>
-      <c r="C3" s="60"/>
-      <c r="D3" s="60"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="60"/>
-      <c r="G3" s="60"/>
-      <c r="H3" s="60"/>
-      <c r="I3" s="60"/>
-      <c r="J3" s="60"/>
-      <c r="K3" s="60"/>
-      <c r="L3" s="60"/>
-      <c r="M3" s="60"/>
-      <c r="N3" s="60"/>
-      <c r="O3" s="60"/>
-      <c r="P3" s="60"/>
-      <c r="Q3" s="60"/>
-      <c r="R3" s="60"/>
-      <c r="S3" s="60"/>
+      <c r="B3" s="62"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="62"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="62"/>
+      <c r="G3" s="62"/>
+      <c r="H3" s="62"/>
+      <c r="I3" s="62"/>
+      <c r="J3" s="62"/>
+      <c r="K3" s="62"/>
+      <c r="L3" s="62"/>
+      <c r="M3" s="62"/>
+      <c r="N3" s="62"/>
+      <c r="O3" s="62"/>
+      <c r="P3" s="62"/>
+      <c r="Q3" s="62"/>
+      <c r="R3" s="62"/>
+      <c r="S3" s="62"/>
       <c r="X3" t="s">
         <v>51</v>
       </c>
@@ -3105,32 +3129,32 @@
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" s="23"/>
-      <c r="B4" s="56" t="s">
+      <c r="B4" s="58" t="s">
         <v>5</v>
       </c>
       <c r="C4" s="39"/>
       <c r="D4" s="39"/>
-      <c r="E4" s="56" t="s">
+      <c r="E4" s="58" t="s">
         <v>7</v>
       </c>
       <c r="F4" s="39"/>
       <c r="G4" s="39"/>
-      <c r="H4" s="56" t="s">
+      <c r="H4" s="58" t="s">
         <v>9</v>
       </c>
       <c r="I4" s="39"/>
       <c r="J4" s="39"/>
-      <c r="K4" s="56" t="s">
+      <c r="K4" s="58" t="s">
         <v>11</v>
       </c>
       <c r="L4" s="39"/>
       <c r="M4" s="39"/>
-      <c r="N4" s="56" t="s">
+      <c r="N4" s="58" t="s">
         <v>13</v>
       </c>
       <c r="O4" s="39"/>
       <c r="P4" s="39"/>
-      <c r="Q4" s="56" t="s">
+      <c r="Q4" s="58" t="s">
         <v>15</v>
       </c>
       <c r="R4" s="39"/>
@@ -3766,27 +3790,27 @@
       </c>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="A13" s="57" t="s">
+      <c r="A13" s="59" t="s">
         <v>55</v>
       </c>
-      <c r="B13" s="58"/>
-      <c r="C13" s="58"/>
-      <c r="D13" s="58"/>
-      <c r="E13" s="58"/>
-      <c r="F13" s="58"/>
-      <c r="G13" s="58"/>
-      <c r="H13" s="58"/>
-      <c r="I13" s="58"/>
-      <c r="J13" s="58"/>
-      <c r="K13" s="58"/>
-      <c r="L13" s="58"/>
-      <c r="M13" s="58"/>
-      <c r="N13" s="58"/>
-      <c r="O13" s="58"/>
-      <c r="P13" s="58"/>
-      <c r="Q13" s="58"/>
-      <c r="R13" s="58"/>
-      <c r="S13" s="58"/>
+      <c r="B13" s="60"/>
+      <c r="C13" s="60"/>
+      <c r="D13" s="60"/>
+      <c r="E13" s="60"/>
+      <c r="F13" s="60"/>
+      <c r="G13" s="60"/>
+      <c r="H13" s="60"/>
+      <c r="I13" s="60"/>
+      <c r="J13" s="60"/>
+      <c r="K13" s="60"/>
+      <c r="L13" s="60"/>
+      <c r="M13" s="60"/>
+      <c r="N13" s="60"/>
+      <c r="O13" s="60"/>
+      <c r="P13" s="60"/>
+      <c r="Q13" s="60"/>
+      <c r="R13" s="60"/>
+      <c r="S13" s="60"/>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A14" s="27" t="s">
@@ -4048,30 +4072,30 @@
       </c>
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A33" s="54" t="s">
+      <c r="A33" s="56" t="s">
         <v>64</v>
       </c>
-      <c r="B33" s="55"/>
-      <c r="C33" s="55"/>
-      <c r="D33" s="55"/>
-      <c r="E33" s="55"/>
-      <c r="F33" s="55"/>
-      <c r="G33" s="55"/>
-      <c r="H33" s="55"/>
-      <c r="I33" s="55"/>
-      <c r="J33" s="55"/>
-      <c r="K33" s="55"/>
-      <c r="L33" s="55"/>
-      <c r="M33" s="55"/>
-      <c r="N33" s="55"/>
-      <c r="O33" s="55"/>
-      <c r="P33" s="55"/>
-      <c r="Q33" s="55"/>
-      <c r="R33" s="55"/>
-      <c r="S33" s="55"/>
+      <c r="B33" s="57"/>
+      <c r="C33" s="57"/>
+      <c r="D33" s="57"/>
+      <c r="E33" s="57"/>
+      <c r="F33" s="57"/>
+      <c r="G33" s="57"/>
+      <c r="H33" s="57"/>
+      <c r="I33" s="57"/>
+      <c r="J33" s="57"/>
+      <c r="K33" s="57"/>
+      <c r="L33" s="57"/>
+      <c r="M33" s="57"/>
+      <c r="N33" s="57"/>
+      <c r="O33" s="57"/>
+      <c r="P33" s="57"/>
+      <c r="Q33" s="57"/>
+      <c r="R33" s="57"/>
+      <c r="S33" s="57"/>
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A34" s="43" t="s">
+      <c r="A34" s="45" t="s">
         <v>65</v>
       </c>
       <c r="B34" s="39"/>
@@ -4452,7 +4476,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="41" t="s">
         <v>74</v>
       </c>
       <c r="B1" s="39"/>
@@ -4464,7 +4488,7 @@
       <c r="H1" s="39"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="62" t="s">
+      <c r="A2" s="40" t="s">
         <v>75</v>
       </c>
       <c r="B2" s="39"/>
@@ -4476,7 +4500,7 @@
       <c r="H2" s="39"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="38" t="s">
         <v>76</v>
       </c>
       <c r="B3" s="39"/>
@@ -4576,19 +4600,19 @@
       </c>
       <c r="C11" s="13">
         <f>IF('Rekap Nilai'!C5&lt;=5,IF('Rekap Nilai'!C5&lt;=1,1,IF('Rekap Nilai'!C5&lt;=2,1,IF('Rekap Nilai'!C5&lt;=3,2,IF('Rekap Nilai'!C5&lt;=4,3,4)))),MAX(0,'Rekap Nilai'!C5-5))*$A$7+IF('Rekap Nilai'!D5&lt;=5,IF('Rekap Nilai'!D5&lt;=1,1,IF('Rekap Nilai'!D5&lt;=2,1,IF('Rekap Nilai'!D5&lt;=3,2,IF('Rekap Nilai'!D5&lt;=4,3,4)))),MAX(0,'Rekap Nilai'!D5-5))*$B$7+IF('Rekap Nilai'!E5&lt;=5,IF('Rekap Nilai'!E5&lt;=1,1,IF('Rekap Nilai'!E5&lt;=2,1,IF('Rekap Nilai'!E5&lt;=3,2,IF('Rekap Nilai'!E5&lt;=4,3,4)))),MAX(0,'Rekap Nilai'!E5-5))*$C$7+IF('Rekap Nilai'!F5&lt;=5,IF('Rekap Nilai'!F5&lt;=1,1,IF('Rekap Nilai'!F5&lt;=2,1,IF('Rekap Nilai'!F5&lt;=3,2,IF('Rekap Nilai'!F5&lt;=4,3,4)))),MAX(0,'Rekap Nilai'!F5-5))*$D$7+IF('Rekap Nilai'!G5&lt;=5,IF('Rekap Nilai'!G5&lt;=1,1,IF('Rekap Nilai'!G5&lt;=2,1,IF('Rekap Nilai'!G5&lt;=3,2,IF('Rekap Nilai'!G5&lt;=4,3,4)))),MAX(0,'Rekap Nilai'!G5-5))*$E$7+IF('Rekap Nilai'!H5&lt;=5,IF('Rekap Nilai'!H5&lt;=1,1,IF('Rekap Nilai'!H5&lt;=2,1,IF('Rekap Nilai'!H5&lt;=3,2,IF('Rekap Nilai'!H5&lt;=4,3,4)))),MAX(0,'Rekap Nilai'!H5-5))*$F$7</f>
-        <v>26.411764705882351</v>
+        <v>26.823529411764707</v>
       </c>
       <c r="D11" s="13">
         <f>IF('Rekap Nilai'!C5&lt;=5,'Rekap Nilai'!C5,'Rekap Nilai'!C5)*$A$7+IF('Rekap Nilai'!D5&lt;=5,'Rekap Nilai'!D5,'Rekap Nilai'!D5)*$B$7+IF('Rekap Nilai'!E5&lt;=5,'Rekap Nilai'!E5,'Rekap Nilai'!E5)*$C$7+IF('Rekap Nilai'!F5&lt;=5,'Rekap Nilai'!F5,'Rekap Nilai'!F5)*$D$7+IF('Rekap Nilai'!G5&lt;=5,'Rekap Nilai'!G5,'Rekap Nilai'!G5)*$E$7+IF('Rekap Nilai'!H5&lt;=5,'Rekap Nilai'!H5,'Rekap Nilai'!H5)*$F$7</f>
-        <v>28.588235294117649</v>
+        <v>28.745098039215687</v>
       </c>
       <c r="E11" s="13">
         <f>IF('Rekap Nilai'!C5&lt;=5,IF('Rekap Nilai'!C5&lt;=1,2,IF('Rekap Nilai'!C5&lt;=2,3,IF('Rekap Nilai'!C5&lt;=3,4,IF('Rekap Nilai'!C5&lt;=4,5,5)))),MIN(100,'Rekap Nilai'!C5+5))*$A$7+IF('Rekap Nilai'!D5&lt;=5,IF('Rekap Nilai'!D5&lt;=1,2,IF('Rekap Nilai'!D5&lt;=2,3,IF('Rekap Nilai'!D5&lt;=3,4,IF('Rekap Nilai'!D5&lt;=4,5,5)))),MIN(100,'Rekap Nilai'!D5+5))*$B$7+IF('Rekap Nilai'!E5&lt;=5,IF('Rekap Nilai'!E5&lt;=1,2,IF('Rekap Nilai'!E5&lt;=2,3,IF('Rekap Nilai'!E5&lt;=3,4,IF('Rekap Nilai'!E5&lt;=4,5,5)))),MIN(100,'Rekap Nilai'!E5+5))*$C$7+IF('Rekap Nilai'!F5&lt;=5,IF('Rekap Nilai'!F5&lt;=1,2,IF('Rekap Nilai'!F5&lt;=2,3,IF('Rekap Nilai'!F5&lt;=3,4,IF('Rekap Nilai'!F5&lt;=4,5,5)))),MIN(100,'Rekap Nilai'!F5+5))*$D$7+IF('Rekap Nilai'!G5&lt;=5,IF('Rekap Nilai'!G5&lt;=1,2,IF('Rekap Nilai'!G5&lt;=2,3,IF('Rekap Nilai'!G5&lt;=3,4,IF('Rekap Nilai'!G5&lt;=4,5,5)))),MIN(100,'Rekap Nilai'!G5+5))*$E$7+IF('Rekap Nilai'!H5&lt;=5,IF('Rekap Nilai'!H5&lt;=1,2,IF('Rekap Nilai'!H5&lt;=2,3,IF('Rekap Nilai'!H5&lt;=3,4,IF('Rekap Nilai'!H5&lt;=4,5,5)))),MIN(100,'Rekap Nilai'!H5+5))*$F$7</f>
-        <v>30.470588235294116</v>
+        <v>30.882352941176471</v>
       </c>
       <c r="F11" s="36">
         <f t="shared" ref="F11:F20" si="0">(C11+D11+E11)/3</f>
-        <v>28.490196078431371</v>
+        <v>28.816993464052288</v>
       </c>
       <c r="G11" s="37">
         <f t="shared" ref="G11:G20" si="1">IF(B11="","",RANK(F11,$F$11:$F$20,0))</f>

</xml_diff>